<commit_message>
Leads: 2026-09-17 00:04 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://www.ciscoheating.com/st-charles-mo-heating-air-conditioning-contractor/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>officeciscoheating@gmail.com</t>
@@ -614,6 +613,62 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Double O Plumbing |</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>doubleoplumbing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://doubleoplumbing.com/emergency-plumbing/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>oscarz@doubleoplumbing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>213-808-2375</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>emergency plumber Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:06 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,6 @@
           <t>https://doubleoplumbing.com/emergency-plumbing/</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>oscarz@doubleoplumbing.com</t>
@@ -669,6 +668,58 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>nothingbutseweranddrains.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://nothingbutseweranddrains.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>nothingbutsewer@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(385) 446-8883</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>West Jordan UT</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>76</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>drain cleaning service West Jordan UT</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:10 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -674,7 +674,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Plumbing</t>
@@ -690,7 +689,6 @@
           <t>https://nothingbutseweranddrains.com/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>nothingbutsewer@gmail.com</t>
@@ -720,6 +718,302 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sewer Repair | WaterHouse Plumbing | New York City, NY</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>waterhouse.nyc</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.waterhouse.nyc/sewer-repair</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>At Waterhouse</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>waterhousecompany@gmail.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(212) 777-3003</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>sewer repair New York NY</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sonoran Ridge Roofing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>roofreplacementgilbert.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://roofreplacementgilbert.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Yes No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>onestopshop@gilbertaz.gov</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(928) 585-0187</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>roof replacement Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Absolute Services</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>absoluteservices.net</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://absoluteservices.net/drain/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>officeservices@absoluteservices.net</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(502) 688-8464</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>sewer repair Louisville KY</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Plumbing NYC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>plumbingnyc.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://plumbingnyc.com/sewer-line-repair-replacement/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@plumbingnyc.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>6465807524</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>New York NY</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>sewer repair New York NY</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Roofing contractor Billings MT</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>bigskycontractors.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://bigskycontractors.com/roofing-contractor-billings-mt/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Results At</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@bigskycontractors.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(406) 313-2829</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>86</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor Billings MT</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:11 UTC (cycle 158)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -864,7 +864,6 @@
           <t>https://absoluteservices.net/drain/sewer-line-repair/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>officeservices@absoluteservices.net</t>
@@ -1014,6 +1013,118 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>EA Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>eaheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.eaheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>eaheatingandcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(915) 691-5394</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>El Paso TX</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>heating and cooling company El Paso TX</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HVAC El Paso</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>deltatheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://deltatheatingandcooling.com/hvac-company-el-paso/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>contact@deltatheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(915)255-9653</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>El Paso TX</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>heating and cooling company El Paso TX</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:14 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1039,7 +1039,6 @@
           <t>https://www.eaheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>eaheatingandcooling@gmail.com</t>
@@ -1095,7 +1094,6 @@
           <t>https://deltatheatingandcooling.com/hvac-company-el-paso/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>contact@deltatheatingandcooling.com</t>
@@ -1125,6 +1123,62 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Fort Wayne Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rickssewerservicefw.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://rickssewerservicefw.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@rickssewerservicefw.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(260) 241-5064</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>84</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>drain cleaning service Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:16 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1149,7 +1149,6 @@
           <t>https://rickssewerservicefw.com/</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>info@rickssewerservicefw.com</t>
@@ -1179,6 +1178,66 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Torrance CA Drain Cleaning Pros</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>draincleaningtorranceca.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://draincleaningtorranceca.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Problems We</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>sohaibsyed880@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(310) 340-1545</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>drain cleaning service Torrance CA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:20 UTC (cycle 164)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1243,6 +1243,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Davis Air Conditioning &amp; Heating, Inc.</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>davisac.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://davisac.com/service-area/air-conditioning-heating-katy-tx</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>For Katy</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>cs.air.conditioning@tdlr.texas.gov</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(281) 410-1153</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>air conditioning repair Katy TX</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:22 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1303,6 +1303,66 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Strategic Heating and Air -</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>strategyac.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://strategyac.com/service/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Stuart Macintire</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>stuart@strategyac.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(602) 377-9142</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>furnace repair Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 00:24 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1363,6 +1363,66 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Seven Peaks Heating</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>sevenpeaksheating.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.sevenpeaksheating.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Operator Sonny</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>estimating@sevenpeaksheating.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(541)668-5696</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Bend OR</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>98</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>HVAC contractor Bend OR</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:15 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1423,6 +1423,62 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Coast to Coast Plumbing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>coasttocoastplumbing.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.coasttocoastplumbing.com/services/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>dispatchexperienceplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>310-275-5800</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>drain cleaning service Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:17 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1444,7 +1444,6 @@
           <t>https://www.coasttocoastplumbing.com/services/drain-cleaning/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>dispatchexperienceplumbing@gmail.com</t>
@@ -1474,6 +1473,66 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Roofer | Gary, IN | Bob The Builder, Inc.</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>bobthebuilderinc.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.bobthebuilderinc.com/contact/roofer-service-area/gary-in</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Bob The</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>roofwes@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(219) 299-0136</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Gary IN</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roofer Gary IN</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:24 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1538,6 +1538,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Summit Dearborn Roof Replacement</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>dearbornroofreplacement.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://dearbornroofreplacement.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Summit Dearborn</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@dearbornroofreplacement.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(313) 631-3546</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Dearborn MI</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>roof replacement Dearborn MI</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:25 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1598,6 +1598,66 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Bordner Home Improvement</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>thinkbordner.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.thinkbordner.com/services/roofing/roof-replacement-independence-mo/</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sam Fleenor</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>connect@bordnerinstall.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>816-358-2102</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Independence MO</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roof replacement Independence MO</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:28 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1658,6 +1658,66 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sanborn's Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>sanbornsac.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.sanbornsac.com/service-areas/rancho-cucamonga/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Star Reviews</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>info@sanbornsac.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>909-793-1234</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>heating and cooling company Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:31 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1718,6 +1718,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TMRG - Jared Langley Roofing &amp; Remodel</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>jaredlangley.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://jaredlangley.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Jared Langley</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>office@jaredlangley.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(406) 251-6363</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Missoula MT</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>84</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Missoula MT</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:34 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1778,6 +1778,122 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>My HVAC Tech</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>myhvac.tech</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.myhvac.tech/contractors/arista-air-conditioning-newark</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@myhvac.tech</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(718) 937-1400</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Newark NJ</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>HVAC contractor Newark NJ</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Arrows Home Air</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>arrowshomeair.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.arrowshomeair.com/cooling</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Founder Fernando</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>office@arrowshomeair.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(971) 707-5226</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>90</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>air conditioning repair Salem OR</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:37 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1799,7 +1799,6 @@
           <t>https://www.myhvac.tech/contractors/arista-air-conditioning-newark</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>info@myhvac.tech</t>
@@ -1889,6 +1888,66 @@
         </is>
       </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>OAKRIDGE Roofing</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>oakridgeroofingutah.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://oakridgeroofingutah.com/service-areas/utah-county-ut/lehi/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Claims Proven</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>info@oakridgeroofingutah.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>(385) 472-8428</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Lehi UT</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>100</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>roof replacement Lehi UT</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:39 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1953,6 +1953,66 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KMG Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>kmgplumbingnola.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://kmgplumbingnola.com/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Backflow Service</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>info@kmgplumbingnola.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(504) 296-7913</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>emergency plumber New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:43 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2013,6 +2013,66 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in McKinney, TX | Texas 1st Choice</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>tx1stchoiceheatair.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://tx1stchoiceheatair.com/heating/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>info@1stchoiceheatair.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(469) 678-4726</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>100</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>heat pump installation McKinney TX</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:48 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2073,6 +2073,126 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Trident Plumbing</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>tridentplumbingva.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://tridentplumbingva.com/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Rebecca Meadows</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>info@tridentplumbingva.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>540-642-0023</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>drain cleaning service Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Bradford Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>bradfordheatcool.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://bradfordheatcool.com/furnace-repair-glendale-az</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Bradford Heating</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@bradfordheatcool.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(623) 624-6246</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Glendale AZ</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>furnace repair Glendale AZ</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:56 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2193,6 +2193,66 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>YAZD Mechanical</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>yazdmechanical.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.yazdmechanical.com/ac-installation-alexandria-va/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Recent Posts</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>info@yazdmechanical.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(703) 981-0055</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Alexandria VA</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>AC installation Alexandria VA</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 13:59 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2253,6 +2253,66 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Climate Experts Air, Plumbing &amp; Electric</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>climateexpertsac.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.climateexpertsac.com/service-areas/palm-bay-fl/water-heaters/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Book Online</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>info@climateexpertsac.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(321) 216-2083</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>water heater repair Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:04 UTC (cycle 34)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2313,6 +2313,66 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>HVAC Rescue</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>hvacrescue.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.hvacrescue.com/heat-pump-installation/gary-in</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>My Personal</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>info@cpkhome.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(866) 373-0169</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Gary IN</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>heat pump installation Gary IN</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:07 UTC (cycle 36)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2373,6 +2373,66 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Navarre’s Plumbing | Expert Plumbing Services in Lafayette, LA | Call (337) 962-</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>navarresplumbingofla.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.navarresplumbingofla.com/Plumber-Lafayette-LA</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Residential Plumbing</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>navarresplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(337) 962-8652</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>90</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>plumbing company Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:18 UTC (cycle 44)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2433,6 +2433,66 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>HVAC &amp; Plumbing Services in Middlesex County | Pespisaco</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>pespisaco.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://pespisaco.com/plumbing-heating-cooling-in-lowell-ma/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Pespisa Company</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>linda@pespisaco.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>617-538-5377</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Lowell MA</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>100</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lowell MA</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:23 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2493,6 +2493,126 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Rivertop Roofing</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>rivertoproofing.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.rivertoproofing.com/roof-replacement-atlanta-ga</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Universal Insurance</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>info@rivertoproofing.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(888) 909-5424</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>100</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>roof replacement Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Gaproroofers</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>gaproroofers.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://gaproroofers.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Free Roof</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>admin@gaproroofers.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>(678) 672-8730</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>100</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>roof replacement Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:26 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2613,6 +2613,66 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Roman Roofing il</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>romanroofingil.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.romanroofingil.com/naperville/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Page County</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>info@romanroofingil.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(630)-724-7720</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>100</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>roof replacement Naperville IL</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:33 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2673,6 +2673,66 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MetFab Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>metfabheating.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.metfabheating.com/air-conditioning/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Tim Feuz</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@metfab-heating.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(360) 892-9542</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>90</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>AC installation Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:38 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2733,6 +2733,66 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>At Your Service Roofing</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>atyourserviceroofing.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://atyourserviceroofing.com/roofing-service-areas/roofing-company-champaign-il/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>At Your</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>stinson.clayton@gmail.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>217.273.3548</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Champaign IL</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>roof repair company Champaign IL</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:45 UTC (cycle 62)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2793,6 +2793,66 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Arizona Roofing Company</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>arizonanativeroofing.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://arizonanativeroofing.com/peoria-roofing-contractor/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>President Arizona</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>info@arizonanativeroofing.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>602-348-6559</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Peoria AZ</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>96</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>roofing contractor Peoria AZ</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 14:57 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2853,6 +2853,66 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Residential Roofing Grand Rapids, Michigan</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>roachhomeimprovement.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://roachhomeimprovement.com/roofing/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>West Michigan</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>office@roachhomeimprovement.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(269) 420-6623</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>100</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>residential roofing company Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:03 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2913,6 +2913,62 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Maverick Roofing</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>maverickroofing.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://maverickroofing.com/amarillo-roofing/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Your Roof</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>bruce@maverickroofing.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Amarillo TX</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>76</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>residential roofing company Amarillo TX</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:04 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2944,7 +2944,6 @@
           <t>bruce@maverickroofing.com</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>Amarillo TX</t>
@@ -2964,6 +2963,62 @@
         </is>
       </c>
       <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Alford Plumbing</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>alfordplumbing.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://alfordplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>alfordplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>931-320-4907</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>90</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>plumbing company Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:12 UTC (cycle 80)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2989,7 +2989,6 @@
           <t>https://alfordplumbing.com/</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>alfordplumbing@gmail.com</t>
@@ -3019,6 +3018,66 @@
         </is>
       </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Portland OR Heat Pump Services: Installation, Repair &amp; Replacement | The Heating</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>theheatingspecialist.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://theheatingspecialist.com/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Google Reviews</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>info@theheatingspecialist.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>503-257-7000</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Portland OR</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>100</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>heat pump installation Portland OR</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:13 UTC (cycle 81)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3083,6 +3083,174 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>S.O.S Drain &amp; Sewer Cleaning Services Inc</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>sossewer.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.sossewer.com/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>jeff@sossewer.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(763) 413-4720</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>90</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>drain cleaning service Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Frazier Plumbing</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>frazierplumbingtn.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://frazierplumbingtn.com/johnson-city-plumber/</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>hello@frazierplumbingtn.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(423) 530-3538</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Johnson City TN</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>plumber Johnson City TN</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>70 Best Roofers in Montgomery, Alabama (2026)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>roofersranked.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://roofersranked.com/best-roofers/alabama/montgomery-al</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>For Montgomery</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>matthew@roofersranked.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Montgomery AL</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>86</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>roofer Montgomery AL</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:26 UTC (cycle 90)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3104,7 +3104,6 @@
           <t>https://www.sossewer.com/</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>jeff@sossewer.com</t>
@@ -3160,7 +3159,6 @@
           <t>https://frazierplumbingtn.com/johnson-city-plumber/</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>hello@frazierplumbingtn.com</t>
@@ -3226,7 +3224,6 @@
           <t>matthew@roofersranked.com</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>Montgomery AL</t>
@@ -3246,6 +3243,62 @@
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>HVAC Services | D &amp; R Heating &amp; Air | Lawton, OK</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>dandrheatandair.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>https://www.dandrheatandair.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>donmargot@sbcglobal.net</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(580) 353-7793</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Lawton OK</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>100</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lawton OK</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:28 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3269,7 +3269,6 @@
           <t>https://www.dandrheatandair.com/</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>donmargot@sbcglobal.net</t>
@@ -3299,6 +3298,66 @@
         </is>
       </c>
       <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Speedy Water Heaters</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>speedywaterheatersoc.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://speedywaterheatersoc.com/service-area/orange-county/santa-ana/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>speedywaterheaters1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(949) 745-4450</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>82</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>water heater repair Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:38 UTC (cycle 98)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3363,6 +3363,62 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Metal Roof Lexington</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>metalrooflexington.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://www.metalrooflexington.com/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>moreinfo@metalrooflexington.com</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>866-868-1006</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>96</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lexington KY</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:40 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3384,7 +3384,6 @@
           <t>https://www.metalrooflexington.com/</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>moreinfo@metalrooflexington.com</t>
@@ -3414,6 +3413,122 @@
         </is>
       </c>
       <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Metal Roofing Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.hesterroofing.net</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.hesterroofing.net/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Cost Comparison</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>contact@hesterroofing.net</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(855) 816-6353</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>90</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Metal Roofing Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.jonestilleyroofingcc.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.jonestilleyroofingcc.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>contact@jonestilleyroofingcc.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(855) 816-6353</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>90</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:45 UTC (cycle 103)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3499,7 +3499,6 @@
           <t>https://aberdeen-sd.jonestilleyroofingcc.com/metal-roofing/</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>contact@jonestilleyroofingcc.com</t>
@@ -3529,6 +3528,66 @@
         </is>
       </c>
       <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ViperJet Drain</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>viperjetdrain.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://www.viperjetdrain.com/service-areas/drain-sewer-cleaning-woodbridge-nj</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Message From</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>src@viperjetdrain.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(201) 877-8976</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>74</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>drain cleaning service Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 15:57 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3593,6 +3593,178 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Precise Comfort and Climate Specialists</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>precisecomfort.net</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://precisecomfort.net/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>mail@precisecomfort.net</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>504-273-0522</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>100</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>heating and cooling company New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Salgau Roofing Inc</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>salgauroofing.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://salgauroofing.com/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>nicolai@salgauroofing.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>(419) 691-9641</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Toledo OH</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>90</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>roofing contractor Toledo OH</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Chappelle Roofing Florida</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>chappelleroofing.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://chappelleroofing.com/location/st-petersburg/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Got You</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>office@chappelleroofing.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>(941) 567-6039</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>90</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>roof replacement St Petersburg FL</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:02 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3614,7 +3614,6 @@
           <t>https://precisecomfort.net/</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>mail@precisecomfort.net</t>
@@ -3670,7 +3669,6 @@
           <t>https://salgauroofing.com/</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>nicolai@salgauroofing.com</t>
@@ -3760,6 +3758,118 @@
         </is>
       </c>
       <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>haleroofingconstruction.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://www.haleroofingconstruction.com/</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>tylerhale1107@gmail.com</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(325) 668-3655</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>98</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>roofing contractor Abilene TX</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ATEX Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>atexroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://atexroofingtx.com/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>atexrc@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(325) 698-3000</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>90</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>roofing contractor Abilene TX</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:03 UTC (cycle 115)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3784,7 +3784,6 @@
           <t>https://www.haleroofingconstruction.com/</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>tylerhale1107@gmail.com</t>
@@ -3840,7 +3839,6 @@
           <t>https://atexroofingtx.com/</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>atexrc@yahoo.com</t>
@@ -3870,6 +3868,66 @@
         </is>
       </c>
       <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Perrault Construction</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>perraultconstruction.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://perraultconstruction.com/duluth-mn/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Remodeling See</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>julie@perraultconstruction.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(218)-723-8477</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>roofing contractor Duluth MN</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:08 UTC (cycle 118)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3933,6 +3933,62 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Magic Electric, Plumbing, Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>themagicteam.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.themagicteam.com/boise/drain-services/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>callcenter@themagicteam.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(208) 877-4544</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>94</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>sewer repair Boise ID</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:09 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3954,7 +3954,6 @@
           <t>https://www.themagicteam.com/boise/drain-services/sewer-line-repair/</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>callcenter@themagicteam.com</t>
@@ -3984,6 +3983,62 @@
         </is>
       </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Air Right Heating And Air</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>airrighttx.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://airrighttx.com/tyler-tx/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>jasonm@airrighttx.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>(903) 549-2700</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Tyler TX</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>100</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>air conditioning repair Tyler TX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:19 UTC (cycle 126)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4009,7 +4009,6 @@
           <t>https://airrighttx.com/tyler-tx/</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>jasonm@airrighttx.com</t>
@@ -4039,6 +4038,62 @@
         </is>
       </c>
       <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Filbert Plumbing</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>filbertplumbing.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://filbertplumbing.com/locations/south-carolina/myrtle-beach/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>info@filbertplumbing.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(855) 796-3280</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>100</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>drain cleaning service Myrtle Beach SC</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:27 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4064,7 +4064,6 @@
           <t>https://filbertplumbing.com/locations/south-carolina/myrtle-beach/drain-cleaning</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>info@filbertplumbing.com</t>
@@ -4094,6 +4093,66 @@
         </is>
       </c>
       <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>PerfectHvac AC Repair Miami Lakes</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>perfecthvac.pro</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://perfecthvac.pro/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Team The</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>info@perfecthvac.pro</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(305) 676-7735</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Hialeah FL</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>90</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>air conditioning repair Hialeah FL</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:28 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4158,6 +4158,66 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Hornet</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>hornetroofing.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://hornetroofing.com/roof-types/metal-roof-services/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Southern Colorado</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>roofsby@hornetroofing.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(719) 299-8848</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Pueblo CO</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Pueblo CO</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:30 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4218,6 +4218,182 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Tri-County Roofing</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>tri-countyroofing.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.tri-countyroofing.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Roof Installation</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>service@tri-countyroofing.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>410-875-9671</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>100</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Fick Bros. Roofing &amp; Exterior Remodeling Company |</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>fickbros.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://fickbros.com/roofing-baltimore-md/roof-replacement/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>jjf@fickbros.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(410) 889-5525</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Delmarva Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>delmarvametalroofing.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://delmarvametalroofing.com/metal-roofing-in-baltimore-md/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Read More</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>contact@delmarvametalroofing.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>855-888-3674</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>84</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:37 UTC (cycle 138)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4299,7 +4299,6 @@
           <t>https://fickbros.com/roofing-baltimore-md/roof-replacement/metal-roofing/</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>jjf@fickbros.com</t>
@@ -4389,6 +4388,66 @@
         </is>
       </c>
       <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Patriot Pros | Castle Rock Heating, Cooling, &amp; Plumbing - Patriot Pros</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>patriotpros.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://patriotpros.com/service-areas/arvada/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Actually Reduce</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>customersupport@patriotpros.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>720-897-5559</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Arvada CO</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>100</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>heating and cooling company Arvada CO</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:43 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4453,6 +4453,66 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Dane Roofing</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>danesroofing.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://www.danesroofing.com/roofing-contractor-in-denton-tx/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>At Dane</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>kelly@danesroofing.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>(469) 585-3263</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>90</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>roofing contractor Denton TX</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:44 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4513,6 +4513,66 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Chicago Drain and Sewer Cleaning</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>rooterflush.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://rooterflush.com/chicago-sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Chicago Sewer</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>contact@rooterflush.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>773-563-4543</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Chicago IL</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>100</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>sewer repair Chicago IL</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 16:50 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4573,6 +4573,66 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Alpaca Roofing</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>alpacaroofing.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://alpacaroofing.com/aurora-co/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Inspection With</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>info@alpacaroofing.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>303-409-4116</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>90</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>roofing contractor Aurora CO</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:08 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L72"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4633,6 +4633,66 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Professional Residential Roofing Services in Rapid City, SD | K1 Roofing</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>k1roofinginc.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://www.k1roofinginc.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Ken Fuerst</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>k1roofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>(605) 430-2340</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Rapid City SD</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>residential roofing company Rapid City SD</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:10 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4693,6 +4693,66 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>lacassaplumbing.com</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>lacassaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://lacassaplumbing.com/naperville-sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Water Heater</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>customerservice@lacassaplumbing.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>(630) 880-2126</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>100</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>sewer repair Naperville IL</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:11 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4753,6 +4753,66 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Expert Roof Repair &amp; Replacement in Waterbury, CT | Roof Angels</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>waterbury-ct.roofangels.org</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://waterbury-ct.roofangels.org/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Skylight Repair</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>info@roofangels.org</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>(877) 510-0035</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Waterbury CT</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>80</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>roof repair company Waterbury CT</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:13 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4813,6 +4813,62 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Lubbockroofer</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>lubbockroofer.net</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://www.lubbockroofer.net/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>jordan@madewell-construction.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>806-570-0264</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Lubbock TX</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>90</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lubbock TX</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:19 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4834,7 +4834,6 @@
           <t>https://www.lubbockroofer.net/metal-roofing</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>jordan@madewell-construction.com</t>
@@ -4864,6 +4863,66 @@
         </is>
       </c>
       <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Quick Quality Plumbing</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>quickqualityplumbingutah.com</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://www.quickqualityplumbingutah.com/sandy/</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Quick Quali</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>office@quickqualityplumbingutah.com</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>801-348-3881</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Sandy UT</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>plumbing company Sandy UT</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:25 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4928,6 +4928,66 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Metal Roofing Contractors | New Braunfels, TX | JD Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>jdmetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://www.jdmetalroofing.com/contact/metal-roofing-contractors-service-area/new-braunfels-tx</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Your Property</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>jdmetal76@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(830) 212-4078</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>100</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>metal roofing contractor New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:32 UTC (cycle 175)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L78"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4988,6 +4988,178 @@
         </is>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Trenchless Sewer Pipe Repair McKinney TX | Sewer Line Repair in McKinney</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>mckinneytrenchlesspiperepair.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://mckinneytrenchlesspiperepair.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Eldorado Estates</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>info@mckinneypiperepair.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>877-552-8556</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>100</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>sewer repair McKinney TX</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Rodriguez Roofing</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>rodriguezroof.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://rodriguezroof.com/katy/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Rodriguez Roofing</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>info@rodriguezroofing.net</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(281) 444-5269</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Katy TX</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>100</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>roofer Katy TX</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Roofer in Escondido, CA</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>sequoiaroofing.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://sequoiaroofing.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>info@sequoiaroofing.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Escondido CA</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>82</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>roofer Escondido CA</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:36 UTC (cycle 178)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5129,13 +5129,11 @@
           <t>https://sequoiaroofing.com/</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>info@sequoiaroofing.com</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
           <t>Escondido CA</t>
@@ -5155,6 +5153,66 @@
         </is>
       </c>
       <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Black Ridge Contracting</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>blackridgecontractor.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://blackridgecontractor.com/</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>drew@blackridgecontractor.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(515) 219-4654</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>98</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>roofing contractor Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:39 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5218,6 +5218,66 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair &amp; Replacement in New Orleans | NolaFLow Plumbing</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>nolaflowplumbing.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://nolaflowplumbing.com/sewer-line-repair-new-orleans/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>New Orleans</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>info@nolaflowplumbing.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>(504) 420-8368</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>New Orleans LA</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>90</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>sewer repair New Orleans LA</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:41 UTC (cycle 181)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5278,6 +5278,66 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Bellingham, Lynden, Ferndale Roofing Contractors</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>axiomrfg.net</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://www.axiomrfg.net/</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Axiom Roofing</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>info@axiomrfg.net</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(360) 354-9937</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>84</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>roofing contractor Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:45 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5338,6 +5338,126 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Frisco, TX | Local Experts</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>parishroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://www.parishroofingsolutions.com/frisco-texas-roofer/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>randy@parishroofingdfw.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(214) 227-8488</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>roof replacement Frisco TX</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>CornerStone Roofing &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>cornerstonerestorationco.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://cornerstonerestorationco.com/roof-repair-newark-nj/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>mishellyerovidev@gmail.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>201-771-2121</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Newark NJ</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>98</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>roof repair company Newark NJ</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:48 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5458,6 +5458,66 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>American Heating Cooling</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>americanhcr.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.americanhcr.com/hvac-contractor-missoula-mt</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Services Residential</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>americanhcr@gmail.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>(406) 203-7548</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Missoula MT</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>HVAC contractor Missoula MT</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:51 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5518,6 +5518,66 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>HVAC Contractor, HVAC Services | Gilbert &amp; Scottsdale, AZ | Country Heating &amp; Co</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>countryheatingandcoolingaz.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.countryheatingandcoolingaz.com/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Jamie Lewis</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>countryheatingaz@aol.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(480) 726-6704</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>90</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>heating and cooling company Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 17:55 UTC (cycle 190)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5578,6 +5578,242 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.klinesplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.klinesplumbingservices.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Homeowner My</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>contact@klinesplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(833) 957-0980</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>90</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>emergency plumber Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Emergency Plumbing in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.mcplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.mcplumbinganddrain.com/</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Here Since</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>contact@mcplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(888) 576-6192</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>90</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>emergency plumber Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Repiping &amp; Whole-Home Plumbing in Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.jlcproplumbing.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.jlcproplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>For Aberdeen</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>contact@jlcproplumbing.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(888) 576-6192</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>90</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>emergency plumber Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Aberdeen, SD</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>aberdeen-sd.waytogoplumber.info</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://aberdeen-sd.waytogoplumber.info/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>contact@waytogoplumber.info</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(833) 652-8604</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>90</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>emergency plumber Aberdeen SD</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 18:01 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5779,7 +5779,6 @@
           <t>https://aberdeen-sd.waytogoplumber.info/</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>contact@waytogoplumber.info</t>
@@ -5809,6 +5808,62 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Heating &amp; Cooling in Reading, Wyomissing, Wernersville, Berks County</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>ultimatecomforthc.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.ultimatecomforthc.com/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>quotes@ultimatecomforthc.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>610-750-8314</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Reading PA</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>100</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>heating and cooling company Reading PA</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 18:06 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5834,7 +5834,6 @@
           <t>https://www.ultimatecomforthc.com/</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>quotes@ultimatecomforthc.com</t>
@@ -5864,6 +5863,66 @@
         </is>
       </c>
       <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ForSure Roofing and Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>forsureroofing.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://www.forsureroofing.com/contact-us</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Randy Smith</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>estimating@forsureroofing.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(515) 367-7873</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Des Moines IA</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>90</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Des Moines IA</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 18:08 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5928,6 +5928,66 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Metal Roofing Fort Wayne, IN: Superior Winter Performance Over Asphalt</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>perfectsteelsolutions.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://www.perfectsteelsolutions.com/metal-roofing-fort-wayne-in/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Fort Wayne</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>residential@perfectsteelsolutions.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>(260) 238-1545</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>90</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Wayne IN</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 18:11 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5988,6 +5988,66 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Drain Master NJ</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>drainmasternj.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://drainmasternj.com/drain-cleaning-toms-river-nj/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Toms River</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>drainandsewernj@gmail.com</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>973-355-0890</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>100</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>drain cleaning service Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 18:14 UTC (cycle 203)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6048,6 +6048,66 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Rochester Drain Rite</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>rochesterdrainritemn.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.rochesterdrainritemn.com/drain-cleaning-services-rochester-mn</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>rochesterdrainrite@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(507) 288-2121</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Rochester MN</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>90</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>drain cleaning service Rochester MN</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 19:40 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6108,6 +6108,62 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Bluebonnet Construct</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>bluebonnetheatandair.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://www.bluebonnetheatandair.com/dentontx</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>rachael@bluebonnetheatandair.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(940) 612-9455</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Denton TX</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>100</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>HVAC contractor Denton TX</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 19:43 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6129,7 +6129,6 @@
           <t>https://www.bluebonnetheatandair.com/dentontx</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>rachael@bluebonnetheatandair.com</t>
@@ -6159,6 +6158,122 @@
         </is>
       </c>
       <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>All About Heat &amp; Air</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>allaboutheatandairnc.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://allaboutheatandairnc.com/hvac-in-asheville-nc/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>office@allaboutplumbingnc.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>828-338-2590</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>100</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>heating and cooling company Asheville NC</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>New Rüf</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>newruf.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://newruf.com/locations/san-marcos-roofing/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Mike Winot</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>info@newruf.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>(512) 642-6005</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>90</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>roof repair company San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 19:46 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6184,7 +6184,6 @@
           <t>https://allaboutheatandairnc.com/hvac-in-asheville-nc/</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>office@allaboutplumbingnc.com</t>
@@ -6274,6 +6273,242 @@
         </is>
       </c>
       <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>DeLuca Roofing, LLC</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>delucaroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.delucaroofingllc.com/</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Estimate Bob</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>delucaroofing@comcast.net</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>412-241-1643</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>100</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>residential roofing company Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Alpha Omega Roofing LLC | Roof Repair &amp; Replacement Experts</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>alphaomegaroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://alphaomegaroofingllc.com/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>info@alphaomegaroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>315-535-2288</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Syracuse NY</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>100</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>roof replacement Syracuse NY</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Residential Roofing Contractors Pittsburgh, PA | Dr. Roofer</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>dr-roofer.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.dr-roofer.com/</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>jake@dr-roofer.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(412) 239-8671</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>100</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>residential roofing company Pittsburgh PA</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Contact Senid Plumbing and Heating For Local Plumbing Contractors Serving Queens</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>senidplumbing.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://senidplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Your Source</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>info@senidplumbing.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(718) 445-3710</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Queens NY</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>100</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>plumbing company Queens NY</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 19:47 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6419,7 +6419,6 @@
           <t>https://www.dr-roofer.com/</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>jake@dr-roofer.com</t>
@@ -6509,6 +6508,62 @@
         </is>
       </c>
       <c r="L104" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Pine Belt Heating and Air | Hattiesburg Heating and Air | Pine Belt Heating &amp; Ai</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>pinebeltheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://pinebeltheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>pinebeltair@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>(601) 299-0011</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Hattiesburg MS</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>86</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>heating and cooling company Hattiesburg MS</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 19:50 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6534,7 +6534,6 @@
           <t>https://pinebeltheatingandair.com/</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>pinebeltair@hotmail.com</t>
@@ -6564,6 +6563,122 @@
         </is>
       </c>
       <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>360 Innovations Roofing Company</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>mydfwroofing.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.mydfwroofing.com/metal-roofing-company/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Donovan Clark</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>360roofco@gmail.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>(214)-402-6943</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>100</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Richardson TX</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Kappler Mechanical &amp; Electrical, Inc.</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>kapplermechanical.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://kapplermechanical.com/city/thornton-co/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>info@kapplermechanical.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>720-513-6481</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>90</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>heat pump installation Thornton CO</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 19:51 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6649,7 +6649,6 @@
           <t>https://kapplermechanical.com/city/thornton-co/</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>info@kapplermechanical.com</t>
@@ -6679,6 +6678,66 @@
         </is>
       </c>
       <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Services Columbia | All Clear Pumping &amp; Sewer</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>allclearmidmo.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://www.allclearmidmo.com/columbia</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>How Columbia</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>contact@allclearmo.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(573) 232-2362</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Columbia MO</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>100</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>drain cleaning service Columbia MO</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 19:53 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6743,6 +6743,122 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>ENG Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>engheating.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://engheating.com/residential/water-heaters/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@engheating.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>(330) 929-0121</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Akron OH</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>90</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>water heater repair Akron OH</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Roofing Contractor in Edmond, OK</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>frontlineexteriors.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://frontlineexteriors.com/edmond/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Frontline Exterior</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>email@frontlineexteriors.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>(405) 697-9939</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>78</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>roofing contractor Edmond OK</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:00 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L110"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6764,7 +6764,6 @@
           <t>https://engheating.com/residential/water-heaters/</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>info@engheating.com</t>
@@ -6854,6 +6853,62 @@
         </is>
       </c>
       <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair Salinas Valley - Acme Plumbing</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>goacmeplumbing.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.goacmeplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>service@goacmeplumbing.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>(831) 422-2311</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Salinas CA</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>88</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>sewer repair Salinas CA</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:03 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6879,7 +6879,6 @@
           <t>https://www.goacmeplumbing.com/</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>service@goacmeplumbing.com</t>
@@ -6909,6 +6908,66 @@
         </is>
       </c>
       <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Alexi Ojeda Roofing | Edmond Roofer</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>alexiojedaroofing.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://www.alexiojedaroofing.com/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Alexi Ojeda</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>alexi@alexiojedaroofing.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>405-914-4691</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>100</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>roofer Edmond OK</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:15 UTC (cycle 26)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6973,6 +6973,66 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>3 Kings Roofing and Gutters</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>3kingsroofingandgutters.com</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.3kingsroofingandgutters.com/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Premium Roofing</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>info@3kingsroofingandgutters.com</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>(317) 900-4336</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Fishers IN</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>100</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>roofing contractor Fishers IN</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:18 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7033,6 +7033,66 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>CHS Cooling and Heating Services</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>chscoolingandheating.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://chscoolingandheating.com/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Very Knowledgeable</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>chssatt@gmail.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>(503) 581-6999</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>90</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>heating and cooling company Salem OR</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:19 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7093,6 +7093,62 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Reyes Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>reyesheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.reyesheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>reyes.hvac@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>(240) 485-8713</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Rockville MD</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>90</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>heating and cooling company Rockville MD</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:21 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7114,7 +7114,6 @@
           <t>https://www.reyesheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>reyes.hvac@yahoo.com</t>
@@ -7144,6 +7143,182 @@
         </is>
       </c>
       <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Source 1 Roofing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>source1roofing.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://www.source1roofing.com/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Term Solutions</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>contact@source1roof.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>(702) 682-1131</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>100</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>roofing contractor North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>On Time NJ</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>njplumbingair.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://njplumbingair.com/water-heater-repair-newark-nj/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Counties Served</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>cityservicegroupnj@gmail.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>862-292-9006</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Newark NJ</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>100</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>water heater repair Newark NJ</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ADJ of Stamford | Home</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>adjofstamford.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://www.adjofstamford.com/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>support@mgsites.net</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>203-348-6448</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Stamford CT</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>90</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>AC installation Stamford CT</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:30 UTC (cycle 36)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7289,7 +7289,6 @@
           <t>https://www.adjofstamford.com/</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
           <t>support@mgsites.net</t>
@@ -7319,6 +7318,66 @@
         </is>
       </c>
       <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Magnolia Plumbing</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>magnoliaplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://magnoliaplumbingco.com/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Replacement Learn</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>office@magnoliaplumbingco.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>901-538-8000</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Memphis TN</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>100</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>plumber Memphis TN</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:33 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7383,6 +7383,126 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>T.O. Plumbing Service, LLC.</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>toplumbingservicellc.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://toplumbingservicellc.com/</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>And Beyond</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>ted@toplumbingservicellc.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>910-977-6723</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>100</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>plumber Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Wade Hardin - Wade Hardin Plumbing</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>wadehardinplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.wadehardinplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Best Service</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>shawn.scott@wadehardinplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>(910) 486-0334</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>100</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>plumber Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:34 UTC (cycle 39)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7503,6 +7503,62 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>San Antonio Plumbing</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>saplumbing.net</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://saplumbing.net/</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>general@sanantonioplumbing.co</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>210-521-0198</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>74</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>plumbing company San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:37 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7524,7 +7524,6 @@
           <t>https://saplumbing.net/</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
           <t>general@sanantonioplumbing.co</t>
@@ -7554,6 +7553,122 @@
         </is>
       </c>
       <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Fults Roofing Company</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>fultsroofing.com</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://fultsroofing.com/residential-roofing-round-rock-tx/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>info@fultsroofing.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(512) 383-5133</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>90</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>residential roofing company Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Best Lawton Roofing</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>lawton-roofing.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://lawton-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Pros Offers</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>info@crcroofingok.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(405) 235-6000</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Lawton OK</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>90</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>residential roofing company Lawton OK</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:40 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7579,7 +7579,6 @@
           <t>https://fultsroofing.com/residential-roofing-round-rock-tx/</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>info@fultsroofing.com</t>
@@ -7669,6 +7668,126 @@
         </is>
       </c>
       <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Prestige Heating and Air Company | Charleston SC | HVAC Repair &amp; Installation</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>prestigeheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://prestigeheatingandair.com/summerville/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Rd Goose</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>janice@prestigeheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>(843) 764-0460</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Summerville SC</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>100</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>HVAC contractor Summerville SC</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Triple M Roofing</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>triplemroof.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://triplemroof.com/metal-roofs/</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>triplemroofing@mailprint.net</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>(440) 904-0586</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Youngstown OH</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>96</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Youngstown OH</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:42 UTC (cycle 44)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7793,6 +7793,62 @@
         </is>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Residential, Commercial, 24/7 Emergency HVAC Installation Contractor Rochester, </t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>turnbullheating.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://www.turnbullheating.com/</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>service@turnbullheating.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>585-501-9100</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Rochester NY</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>98</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>AC installation Rochester NY</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:43 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7814,7 +7814,6 @@
           <t>https://www.turnbullheating.com/</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>service@turnbullheating.com</t>
@@ -7844,6 +7843,66 @@
         </is>
       </c>
       <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Miramar Roofing Contractor | AGK Construction &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>agkgc.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://agkgc.com/miramar-roofing</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Roofing Approvals</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>info@agkgc.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>(954)807-3455</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>90</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>roofing contractor Miramar FL</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:48 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7908,6 +7908,66 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>One Hour Heating and Air Conditioning of Mission Viejo</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>onehourheatandairorangecounty.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://www.onehourheatandairorangecounty.com/irvine</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Locally Trusted</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>info@onehourheatandairorangecounty.com</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>949-464-7748</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>90</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>air conditioning repair Irvine CA</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 20:58 UTC (cycle 55)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L129"/>
+  <dimension ref="A1:L130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7968,6 +7968,66 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Medford's Plumbing</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>medfordsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>https://www.medfordsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Installation We</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>info@medfordsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>(934) 732 1047</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Medford OR</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>100</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>emergency plumber Medford OR</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:00 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8028,6 +8028,66 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>abilenerestoration.com</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>abilenerestoration.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://abilenerestoration.com/abilene-roofing/</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Without This</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>abilenerestoration@gmail.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>(325) 370-0320</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Abilene TX</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>100</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>roof replacement Abilene TX</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:03 UTC (cycle 58)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8088,6 +8088,62 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Steve’s Ultimate Air</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>stevesultimateair.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://stevesultimateair.com/ac-repair-peoria/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>stevesultimateair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>(480) 458-7287</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Peoria AZ</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>100</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>air conditioning repair Peoria AZ</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:28 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8109,7 +8109,6 @@
           <t>https://stevesultimateair.com/ac-repair-peoria/</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>stevesultimateair@gmail.com</t>
@@ -8139,6 +8138,62 @@
         </is>
       </c>
       <c r="L132" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Air Conditioning Troy, MI| Furnace Repair Troy, MI</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>mainheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://www.mainheatingandcooling.com/service-area/troy-heating-and-air-conditioning-repair.php</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>service@mainheating.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>586-731-0950</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Troy MI</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>90</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>furnace repair Troy MI</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:34 UTC (cycle 79)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8164,7 +8164,6 @@
           <t>https://www.mainheatingandcooling.com/service-area/troy-heating-and-air-conditioning-repair.php</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>service@mainheating.com</t>
@@ -8194,6 +8193,62 @@
         </is>
       </c>
       <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>EXETR Exteriors | Roofing &amp; Storm Restoration Cary NC</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>exetr.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://exetr.com/roof-replacement-cary-nc</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>office@exetr.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>(919) 717-4032</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Cary NC</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>86</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>roof replacement Cary NC</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:37 UTC (cycle 81)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8219,7 +8219,6 @@
           <t>https://exetr.com/roof-replacement-cary-nc</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>office@exetr.com</t>
@@ -8249,6 +8248,66 @@
         </is>
       </c>
       <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Bon Air Service Company</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>bonairservice.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://bonairservice.com/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Checkups Standard</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>parts@bonairservice.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>972-264-2244</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>90</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>furnace repair Grand Prairie TX</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:38 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8313,6 +8313,118 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Plumbing | Corpus Christi, TX | Double A Plumbing</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>doubleaplumbingcctex.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://doubleaplumbingcctex.com/</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>adriansalazar1123@gmail.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>1361315583</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>100</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>plumbing company Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>C C Anchor Plumbing, Inc. - Home</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>c-c-anchor-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.c-c-anchor-plumbing.com/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>ccanchor@att.net</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>361.937.7555</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>76</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>plumbing company Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:43 UTC (cycle 85)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L137"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8334,7 +8334,6 @@
           <t>https://doubleaplumbingcctex.com/</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
           <t>adriansalazar1123@gmail.com</t>
@@ -8390,7 +8389,6 @@
           <t>https://www.c-c-anchor-plumbing.com/</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
           <t>ccanchor@att.net</t>
@@ -8420,6 +8418,122 @@
         </is>
       </c>
       <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Pioneer Plumbing</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>pioneerplumbing.net</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://pioneerplumbing.net/drain-services/drain-clearing-service/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Schedule Now</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>info@pioneerplumbing.net</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>(520) 499-1421</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>100</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>drain cleaning service Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Welcome to Our Plumbing &amp; Drain Cleaning Services</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>calldrainmedics.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://calldrainmedics.com/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>service@azdrainmedics.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>(520) 675-3574</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>90</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>drain cleaning service Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:45 UTC (cycle 87)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8504,7 +8504,6 @@
           <t>https://calldrainmedics.com/</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>service@azdrainmedics.com</t>
@@ -8534,6 +8533,126 @@
         </is>
       </c>
       <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Triggs Plumbing - Madison, WI</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>triggsplumbingwi.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://www.triggsplumbingwi.com/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Triggs Plumbing</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>triggs@triggsplumbing.net</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>(608) 256-2966</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>96</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>plumber Madison WI</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>HJ Pertzborn</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>hjpertzborn.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://hjpertzborn.com/</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Fire Protection</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>pertzborn@hjpertzborn.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>608-256-3900</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>90</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>plumber Madison WI</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:47 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8658,6 +8658,62 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Superior Roofing and Restoration | Edmond, Oklahoma's Trusted Roofing Experts</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>superiorroofingok.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://superiorroofingok.com/</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>info@superiorroofingok.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>405-972-3501</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>88</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>roof repair company Edmond OK</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:48 UTC (cycle 89)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8679,7 +8679,6 @@
           <t>https://superiorroofingok.com/</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>info@superiorroofingok.com</t>
@@ -8709,6 +8708,66 @@
         </is>
       </c>
       <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Plumbing Contractor | Bloomington, MN | Richfield Plumbing Company</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>richfieldplumbing.com</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://www.richfieldplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>David Adelmann</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>service@richfieldplumbing.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>(952) 881-3355</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Bloomington MN</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>88</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>plumbing company Bloomington MN</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:53 UTC (cycle 92)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L143"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8773,6 +8773,126 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair &amp; Replacement in San Francisco, CA | ASAP Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>asapplumbingpro.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://www.asapplumbingpro.com/sewer-line/san-francisco-ca/</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Why San</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>service@asapplumbingpro.com</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>(415) 728-6391</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>100</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>sewer repair San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Sewer Repair Services in San Francisco, CA | Heise's Plumbing</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>heisesplumbing.com</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://www.heisesplumbing.com/san-francisco/sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Fast Response</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>heisesplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>(415) 333-0704</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>90</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>sewer repair San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 21:57 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8893,6 +8893,66 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Paskar Plumbing, Drains, Water Heaters Brooklyn Park, MN</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>paskarplumbing.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://www.paskarplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Twin Cities</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>paskarplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>612-483-0348</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>90</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>plumber Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:00 UTC (cycle 97)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8953,6 +8953,62 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Cassal Cooling and Heating</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>cassalcoolingheating.com</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://www.cassalcoolingheating.com/</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>john@smith.com</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>(575) 520-5655</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>100</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>heating and cooling company Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:03 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L147"/>
+  <dimension ref="A1:L148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8974,7 +8974,6 @@
           <t>https://www.cassalcoolingheating.com/</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
           <t>john@smith.com</t>
@@ -9004,6 +9003,66 @@
         </is>
       </c>
       <c r="L147" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Reliable HVAC</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>reliablehvactx.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://reliablehvactx.com/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Sugar Land</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>reliablehvac88@gmail.com</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>(832) 781-7283</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>100</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>HVAC contractor Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:12 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L148"/>
+  <dimension ref="A1:L149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9068,6 +9068,62 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Thrive Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>thriveheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://thriveheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>rhys@thriveheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>(360) 502-6561</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Everett WA</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>88</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>heating and cooling company Everett WA</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:13 UTC (cycle 106)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L149"/>
+  <dimension ref="A1:L150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9089,7 +9089,6 @@
           <t>https://thriveheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
           <t>rhys@thriveheatingandcooling.com</t>
@@ -9119,6 +9118,62 @@
         </is>
       </c>
       <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Lion Services LLC</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>lionservicesllc.com</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://lionservicesllc.com/pawtucket-ri/</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>info@lionservicesllc.com</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>(401) 205-8518</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Pawtucket RI</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>80</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>roof repair company Pawtucket RI</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:25 UTC (cycle 114)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L150"/>
+  <dimension ref="A1:L151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9144,7 +9144,6 @@
           <t>https://lionservicesllc.com/pawtucket-ri/</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>info@lionservicesllc.com</t>
@@ -9174,6 +9173,62 @@
         </is>
       </c>
       <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Cool Cat Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>coolcatheating.com</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://coolcatheating.com/services/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>coolcatheating@gmail.com</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>(828) 589-3580</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>100</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>AC installation Asheville NC</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:29 UTC (cycle 117)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L151"/>
+  <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9199,7 +9199,6 @@
           <t>https://coolcatheating.com/services/ac-installation/</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
           <t>coolcatheating@gmail.com</t>
@@ -9229,6 +9228,66 @@
         </is>
       </c>
       <c r="L151" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Quality HVAC Services | High Point NC | Evans Air Services</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>evansairservices.com</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://www.evansairservices.com/high-point--nc</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>High Point</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>evansairservices2@gmail.com</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>(336) 297-9922</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>High Point NC</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>90</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>air conditioning repair High Point NC</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:44 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9293,6 +9293,126 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Mill Creek &amp; Everett Roofers Contractors Repair &amp; Install</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>masterswa.com</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://masterswa.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Chuck Dominguez</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>info@masterswa.com</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>(425) 244-0551</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Everett WA</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>100</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Everett WA</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Jackson Plumbing and Drain Services</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>jackson.plumbingdrainservices.com</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://jackson.plumbingdrainservices.com/</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Jackson Plumbing</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>info@jackson.plumbingdrainservices.com</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>(601) 326-1669</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Jackson MS</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>90</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>plumber Jackson MS</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:47 UTC (cycle 129)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9413,6 +9413,62 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Top-Quality Air Conditioning Sales and Installation | Brooklyn, NY | B &amp; R Elect</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>acservicebrooklyn.com</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://www.acservicebrooklyn.com/air-conditioning-installations</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>brtvacltd@gmail.com</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>(718) 743-2407</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>80</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>AC installation Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 22:48 UTC (cycle 130)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L155"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9434,7 +9434,6 @@
           <t>https://www.acservicebrooklyn.com/air-conditioning-installations</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
           <t>brtvacltd@gmail.com</t>
@@ -9464,6 +9463,126 @@
         </is>
       </c>
       <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Dunzo Roofing &amp; Gutters</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>calldunzo.com</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://calldunzo.com/service-area/concord/</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Submit Why</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>contactus@calldunzo.com</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>704.834.1725</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Concord NC</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>100</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>roofer Concord NC</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Summit Exteriors Inc.</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>summitexteriorsmn.com</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://summitexteriorsmn.com/woodbury/</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Storm Damage</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>info@summitexteriorsmn.com</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>(763) 300-3245</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Woodbury MN</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>90</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>roofing contractor Woodbury MN</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:04 UTC (cycle 141)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L157"/>
+  <dimension ref="A1:L160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9588,6 +9588,174 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>5Star Plumbing Family</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>5starplumbingfamily.com</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://5starplumbingfamily.com/</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Line Launches</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>info@5starplumbingfamily.com</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>(478) 307-7638</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Macon GA</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>90</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>plumbing company Macon GA</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Jacobs Cathey Co. | Waco, Texas HVAC</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>jacobscathey.com</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://www.jacobscathey.com/</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>info@jcac.net</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>(254) 772-9572</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Waco TX</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>88</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>HVAC contractor Waco TX</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>DeBackers Inc | HVAC Contractors | Topeka, KS</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>debackersinc.com</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://www.debackersinc.com/</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>debackerhvac@aol.com</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr"/>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Topeka KS</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>76</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>HVAC contractor Topeka KS</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:14 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L160"/>
+  <dimension ref="A1:L161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9669,7 +9669,6 @@
           <t>https://www.jacobscathey.com/</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
         <is>
           <t>info@jcac.net</t>
@@ -9725,13 +9724,11 @@
           <t>https://www.debackersinc.com/</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
           <t>debackerhvac@aol.com</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr"/>
       <c r="H160" t="inlineStr">
         <is>
           <t>Topeka KS</t>
@@ -9751,6 +9748,66 @@
         </is>
       </c>
       <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Beaverton Roof Pros</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>beavertonroofpros.com</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://beavertonroofpros.com/</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Beaverton Roof</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>quotes@beavertonroofpros.com</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>(971) 298-7833</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Beaverton OR</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>100</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>roof repair company Beaverton OR</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:21 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L161"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9813,6 +9813,122 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Rockford, IL | Pure Flo H2O LLC</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>purefloh2o.com</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://www.purefloh2o.com/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>servicepurefloh2o@gmail.com</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>(815) 242-0992</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>94</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>water heater repair Rockford IL</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Plumbers Rockford</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>plumbersrockford.com</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://plumbersrockford.com/services/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Local Rockford</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>service@plumbersrockford.com</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>(815) 783-0034</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>90</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>water heater repair Rockford IL</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:23 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9834,7 +9834,6 @@
           <t>https://www.purefloh2o.com/water-heater-repair</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
           <t>servicepurefloh2o@gmail.com</t>
@@ -9924,6 +9923,174 @@
         </is>
       </c>
       <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Air Medic HVAC</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>youracdoctor.com</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://youracdoctor.com/</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>info@youracdoctor.com</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>(225) 229-4956</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>100</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>HVAC contractor Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>HVAC Company Baton Rouge, LA</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>acadianheatingair.com</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://acadianheatingair.com/</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>acadianheatingandair@gmail.com</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>225 819 3757</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>90</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>HVAC contractor Baton Rouge LA</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>AC Repair | Clarksville, Tennessee | H&amp;H HVAC</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>hhheating.net</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://www.hhheating.net/ac-repair</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>acservices@hh-heating.com</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>931-358-2600</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>86</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>air conditioning repair Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:29 UTC (cycle 158)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L166"/>
+  <dimension ref="A1:L167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9949,7 +9949,6 @@
           <t>https://youracdoctor.com/</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
           <t>info@youracdoctor.com</t>
@@ -10005,7 +10004,6 @@
           <t>https://acadianheatingair.com/</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
         <is>
           <t>acadianheatingandair@gmail.com</t>
@@ -10061,7 +10059,6 @@
           <t>https://www.hhheating.net/ac-repair</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
           <t>acservices@hh-heating.com</t>
@@ -10091,6 +10088,62 @@
         </is>
       </c>
       <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Sewer Repair Baltimore</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>sewerrepairbaltimore.com</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://www.sewerrepairbaltimore.com/service/sewer_repair.html</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>info@sewerrepairbaltimore.com</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>(888) 602-4224</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>70</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>sewer repair Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:33 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L167"/>
+  <dimension ref="A1:L169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10114,7 +10114,6 @@
           <t>https://www.sewerrepairbaltimore.com/service/sewer_repair.html</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
         <is>
           <t>info@sewerrepairbaltimore.com</t>
@@ -10144,6 +10143,126 @@
         </is>
       </c>
       <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Parma, OH</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>atlasroofingrestoration.com</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://atlasroofingrestoration.com/oh/parma/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Northeast Ohio</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>office@atlasroofingrestoration.com</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>(216) 888-3208</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Parma OH</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>100</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>roof replacement Parma OH</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>FHC</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>franklinheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://www.franklinheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Foster Franklin</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>service@franklinheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>615-790-7208</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Franklin TN</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>88</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>HVAC contractor Franklin TN</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:35 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L169"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10268,6 +10268,62 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Ed's Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>edsroofing.com</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://www.edsroofing.com/</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>edsroof@gmail.com</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>(360) 687-2963</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>90</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>roofer Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:38 UTC (cycle 164)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L170"/>
+  <dimension ref="A1:L172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10289,7 +10289,6 @@
           <t>https://www.edsroofing.com/</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr">
         <is>
           <t>edsroof@gmail.com</t>
@@ -10319,6 +10318,122 @@
         </is>
       </c>
       <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Dr. Roof Inc.</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>drroofinc.com</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://drroofinc.com/residential-roofing-vancouver-wa/</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>drroofinc1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>(360) 852-8884</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>98</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>residential roofing company Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>J&amp;P Roofing &amp; Construction Inc.</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>jnproofing.net</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://jnproofing.net/residential-roofing</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Malarkey Certified</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>office@jnproofing.net</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>360-901-6905</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>90</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>residential roofing company Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:47 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L172"/>
+  <dimension ref="A1:L174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10344,7 +10344,6 @@
           <t>https://drroofinc.com/residential-roofing-vancouver-wa/</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
           <t>drroofinc1@gmail.com</t>
@@ -10434,6 +10433,118 @@
         </is>
       </c>
       <c r="L172" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>L &amp; R Heating &amp; Air Conditioning, Inc</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>lrhvacinc.com</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://www.lrhvacinc.com/services/repair/</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>jw@lrhvacinc.com</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>310-328-1209</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>100</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>furnace repair Torrance CA</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Lovotti Inc</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>lovottiinc.com</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://lovottiinc.com/</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>admin@lovottiinc.com</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>(209) 931-2100</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>94</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>HVAC contractor Stockton CA</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:49 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L174"/>
+  <dimension ref="A1:L175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10459,7 +10459,6 @@
           <t>https://www.lrhvacinc.com/services/repair/</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
           <t>jw@lrhvacinc.com</t>
@@ -10515,7 +10514,6 @@
           <t>https://lovottiinc.com/</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
           <t>admin@lovottiinc.com</t>
@@ -10545,6 +10543,62 @@
         </is>
       </c>
       <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Guardian Tempe Heating and Cooling â Professional HVAC Repair &amp; Installation i</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>guardiantempeheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>http://guardiantempeheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>salem@guardiantempeheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>(480) 542-8143</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Tempe AZ</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>78</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>heating and cooling company Tempe AZ</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:51 UTC (cycle 173)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L175"/>
+  <dimension ref="A1:L176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10569,7 +10569,6 @@
           <t>http://guardiantempeheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
           <t>salem@guardiantempeheatingandcooling.com</t>
@@ -10599,6 +10598,66 @@
         </is>
       </c>
       <c r="L175" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Tight Fit Plumbing</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>tightfitplumbing.com</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://tightfitplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Online Reliable</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>sales@tightfitplumbing.com</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>9134555051</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>100</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>plumber Olathe KS</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
         <is>
           <t>2026-09-17</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:52 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L176"/>
+  <dimension ref="A1:L177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10663,6 +10663,66 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Robinhood Exterior - Trusted Roofing Contractor in Elkton, MD</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>robinhoodexterior.com</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://robinhoodexterior.com/roof-replacement-in-newark-de/</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Vision Our</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>josh@rhexterior.com</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>410-538-1970</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Newark DE</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>90</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>roof replacement Newark DE</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-17 23:54 UTC (cycle 175)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-17.xlsx
+++ b/output/leads_2026-09-17.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L177"/>
+  <dimension ref="A1:L178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10723,6 +10723,62 @@
         </is>
       </c>
     </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Prime Flow Plumbing</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>primeflowplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://primeflowplumbingllc.com/west-jordan-ut/</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>service@primeflowplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>(385) 332-3900</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>West Jordan UT</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>90</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>plumbing company West Jordan UT</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>